<commit_message>
fix: resolver error de carga en cronograma y evitar bloqueo en edicion de sede de usuario
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_tecnicos.xlsx
+++ b/public/templates/plantilla_tecnicos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeanp\Documents\registro\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B60B362-AB31-4EC1-9F81-170C833CCA4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203C4003-3412-476C-8DD0-506F820C2AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Nombre Completo</t>
   </si>
@@ -32,48 +32,6 @@
   </si>
   <si>
     <t>Sede (Opcional)</t>
-  </si>
-  <si>
-    <t>TECNICO</t>
-  </si>
-  <si>
-    <t>Campus Villa</t>
-  </si>
-  <si>
-    <t>Sebastian Gabriel, Puma Beltran</t>
-  </si>
-  <si>
-    <t>Jean Pieer Pinchi Bernuy Ortiz</t>
-  </si>
-  <si>
-    <t>Maycol Javier Palacios Pesantes</t>
-  </si>
-  <si>
-    <t>Kevin Jesus Muñoz Nieto</t>
-  </si>
-  <si>
-    <t>German Elias Flores Ybala</t>
-  </si>
-  <si>
-    <t>José Humberto Calderon Castro</t>
-  </si>
-  <si>
-    <t>Miguel Angel Quispe Estrella</t>
-  </si>
-  <si>
-    <t>Juan Manuel Torvisco Tuesta</t>
-  </si>
-  <si>
-    <t>Campus Ate</t>
-  </si>
-  <si>
-    <t>Hugo Cruz Rengifo</t>
-  </si>
-  <si>
-    <t>00119519</t>
-  </si>
-  <si>
-    <t>Campus Norte</t>
   </si>
 </sst>
 </file>
@@ -114,7 +72,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,35 +80,24 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,7 +446,7 @@
     <col min="4" max="4" width="14.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.2" thickBot="1">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,143 +460,55 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2">
-        <v>81161551</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="2">
-        <v>72455873</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2">
-        <v>46269338</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2">
-        <v>49074636</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2">
-        <v>42102991</v>
-      </c>
-      <c r="C6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="3">
-        <v>43658704</v>
-      </c>
-      <c r="C7" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="2">
-        <v>41021521</v>
-      </c>
-      <c r="C8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="2">
-        <v>41704513</v>
-      </c>
-      <c r="C9" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="16.2" thickBot="1">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="16.2" thickBot="1">
+    <row r="2" spans="1:4">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="1"/>
+      <c r="B3" s="2"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1"/>
+      <c r="B6" s="6"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1"/>
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1"/>
+      <c r="B8" s="2"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1"/>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" ht="16.2" thickBot="1">
+      <c r="B11" s="4"/>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="1"/>
+      <c r="B12" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 C2:D2 C3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>